<commit_message>
Brand the order email and PDF, and fix cart totals and sheet notify.
Quote sheets now use real line quantities, and submit no longer depends on a silent phone invoke.
</commit_message>
<xml_diff>
--- a/docs/import-template.xlsx
+++ b/docs/import-template.xlsx
@@ -9,8 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fitment" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parts'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fitment'!$A$1:$D$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,16 +30,40 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B2C5B"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B2C5B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF7E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F6F8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +71,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D5DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D5DD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D5DD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D5DD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -123,6 +171,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SSG</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>Yellow rows are examples. Keep adding new SKUs in the grey rows below. Do not change the header names.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>SSG</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>Blank Model = all models of that Make. Blank Variant = all variants of that Model.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -414,166 +492,588 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Name_UR</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>OEM_Number</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Price_PKR</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Description_UR</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Image_Filename</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>SSG-BRK-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Front Brake Pad Set</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>فرنٹ بریک پیڈ سیٹ</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Brembo</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>04465-YZZE1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>brakes</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="2" t="n">
         <v>7200</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Ceramic front pads for Corolla GLi.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>کرولا جی ایل آئی کے لیے فرنٹ سیرامک پیڈز۔</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="b">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SSG-BRK-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Front Brake Pad Set</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>فرنٹ بریک پیڈ سیٹ</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Brembo</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>45022-TR0-A00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>brakes</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>8100</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Front pads for Civic Oriel.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>سوک اوریئل کے لیے فرنٹ پیڈز۔</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>SSG-FLT-001</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Oil Filter</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>آئل فلٹر</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Denso</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>90915-YZZD2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>filters</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="G4" s="2" t="n">
         <v>950</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Spin-on oil filter for all Corolla variants.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>تمام کرولا ویرینٹس کے لیے آئل فلٹر۔</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="b">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="b">
         <v>1</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SSG-ENG-001</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Iridium Spark Plug (set of 4)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>ایریڈیم اسپارک پلگ (4)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>NGK</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>90919-01253</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>4200</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Iridium plugs for Corolla 1.6/1.8.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>کرولا 1.6/1.8 کے لیے ایریڈیم پلگ۔</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SSG-ELC-001</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Battery 60Ah</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>بیٹری 60 ایمپئیر</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Amaron</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>28800-0L040</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>electrical</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>18500</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Maintenance-free 60Ah battery.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>60 ایمپئیر مینٹیننس فری بیٹری۔</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr"/>
+      <c r="K18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr"/>
+      <c r="K22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+      <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -583,88 +1083,444 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Make</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Variant</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>SSG-BRK-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Toyota</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Corolla</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>GLi</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SSG-BRK-001</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Corolla</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SSG-BRK-002</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Honda</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Civic</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Oriel</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SSG-FLT-001</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Corolla</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SSG-ENG-001</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Corolla</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SSG-ELC-001</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr"/>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr"/>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr"/>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr"/>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr"/>
+      <c r="B36" s="3" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr"/>
+      <c r="B37" s="3" t="inlineStr"/>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>SSG catalogue import template</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SSG-BRK-001</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Toyota</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Corolla</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>How to fill</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SSG-FLT-001</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Toyota</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Corolla</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>1. Keep the sheet names exactly: Parts and Fitment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2. Yellow rows are samples. Copy that pattern into the grey empty rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3. Do not add Rs or commas in Price_PKR. Use 7200 not Rs 7,200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4. Category must be one of: brakes, filters, engine, electrical, suspension, cooling, lighting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5. Active: TRUE or FALSE. Leave blank for TRUE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6. Fitment SKU must match a SKU on the Parts sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>7. Leave Model blank to mean all models of that make.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8. Leave Variant blank to mean all variants of that model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9. Save as .xlsx and upload from Admin → Catalogue import.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Required Parts columns: SKU, Name, Category, Price_PKR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Required Fitment columns: SKU, Make</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>